<commit_message>
demo: alinha id_datajuri (10683/12175/11839) entre demo_seed e planilha do agente
Sem isso o POST /api/robo/resultado dava 404 e o alerta cross-produto não
aparecia na web. Verificado end-to-end com servidor real + agente (MODO_SIMULADO):
alerta chega, tarefa não duplica.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/agente-eproc/planilha_exemplo.xlsx
+++ b/agente-eproc/planilha_exemplo.xlsx
@@ -436,7 +436,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CLI-001</t>
+          <t>10683</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -453,7 +453,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>CLI-002</t>
+          <t>12175</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -470,7 +470,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CLI-003</t>
+          <t>11839</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -487,7 +487,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CLI-004</t>
+          <t>100204</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">

</xml_diff>